<commit_message>
added verification steps and created folder
</commit_message>
<xml_diff>
--- a/docs/26_Validation_Timing_Checklist.xlsx
+++ b/docs/26_Validation_Timing_Checklist.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'How to Use'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Gate Summary'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Build Checklist'!$A$4:$K$600</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Build Checklist'!$A$4:$L$600</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Build Checklist'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Build Checklist'!$A$1:$K$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Re-validation Log'!$A$4:$I$300</definedName>
@@ -33,7 +33,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -171,6 +171,12 @@
       <color rgb="FF404040"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <color rgb="FF0563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -265,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -430,6 +436,18 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -870,7 +888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -980,7 +998,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>When a row carries a Suite number, the column beside it says “Yes — check n”. Record that result in document 22 as well, on the Check Results tab, against the same check. Doc 22 is the formal record of the seventeen; this workbook is the working tick-list.</t>
+          <t>When a row carries a Suite number, the column beside it says “Yes — check n”. Record that result in document 22 as well, on the Check Results tab, against the same check. Doc 22 is the formal record of the seventeen; this workbook is the working tick-list. The Procedure column on the same row names the step-by-step document for that check in docs/validation/ — open it if you have not run the check before.</t>
         </is>
       </c>
     </row>
@@ -1179,6 +1197,18 @@
       <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Development Checklist — the build tasks. Its phases map to the gates: G0 = Phases 0–1, G1 = 2, G2 = 3, G3 = 4, G4 = 5, G5 = 6, G6 = 7, G7 and G8 = 8, G9 = 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>docs/validation/</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>One step-by-step procedure per suite check, V01 to V17, in .docx and .xlsx. The Procedure column on the Build Checklist names the one that covers each row.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K600"/>
+  <dimension ref="A1:L600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1858,6 +1888,7 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1870,7 +1901,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>The recording companion to document 25. Work down the gates in order and set Result on every row; the Gate Summary tab counts itself from this column. A row with a Suite number is also recorded in document 22 against the same check. A gate is PASSED when every row is Pass or N/A.</t>
+          <t>The recording companion to document 25. Work down the gates in order and set Result on every row; the Gate Summary tab counts itself from this column. A row with a Suite number is also recorded in document 22 against the same check. A gate is PASSED when every row is Pass or N/A. The Procedure column names the step-by-step document for that check in docs/validation/ — one file per check, V01 to V17.</t>
         </is>
       </c>
     </row>
@@ -1928,6 +1959,11 @@
       <c r="K4" s="34" t="inlineStr">
         <is>
           <t>Observed value / notes</t>
+        </is>
+      </c>
+      <c r="L4" s="34" t="inlineStr">
+        <is>
+          <t>Procedure</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1982,8 @@
       <c r="H5" s="36" t="n"/>
       <c r="I5" s="36" t="n"/>
       <c r="J5" s="36" t="n"/>
-      <c r="K5" s="37" t="n"/>
+      <c r="K5" s="36" t="n"/>
+      <c r="L5" s="37" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="38" t="inlineStr">
@@ -2083,7 +2120,8 @@
       <c r="H9" s="36" t="n"/>
       <c r="I9" s="36" t="n"/>
       <c r="J9" s="36" t="n"/>
-      <c r="K9" s="37" t="n"/>
+      <c r="K9" s="36" t="n"/>
+      <c r="L9" s="37" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="38" t="inlineStr">
@@ -2286,6 +2324,11 @@
       <c r="I14" s="43" t="n"/>
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="15" t="n"/>
+      <c r="L14" s="59" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="44" t="inlineStr">
@@ -2328,6 +2371,11 @@
       <c r="I15" s="50" t="n"/>
       <c r="J15" s="23" t="n"/>
       <c r="K15" s="22" t="n"/>
+      <c r="L15" s="60" t="inlineStr">
+        <is>
+          <t>V12</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="38" t="inlineStr">
@@ -2424,7 +2472,8 @@
       <c r="H18" s="36" t="n"/>
       <c r="I18" s="36" t="n"/>
       <c r="J18" s="36" t="n"/>
-      <c r="K18" s="37" t="n"/>
+      <c r="K18" s="36" t="n"/>
+      <c r="L18" s="37" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="38" t="inlineStr">
@@ -2507,6 +2556,11 @@
       <c r="I20" s="50" t="n"/>
       <c r="J20" s="23" t="n"/>
       <c r="K20" s="22" t="n"/>
+      <c r="L20" s="60" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="38" t="inlineStr">
@@ -2589,6 +2643,11 @@
       <c r="I22" s="50" t="n"/>
       <c r="J22" s="23" t="n"/>
       <c r="K22" s="22" t="n"/>
+      <c r="L22" s="60" t="inlineStr">
+        <is>
+          <t>V05</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="38" t="inlineStr">
@@ -2685,7 +2744,8 @@
       <c r="H25" s="36" t="n"/>
       <c r="I25" s="36" t="n"/>
       <c r="J25" s="36" t="n"/>
-      <c r="K25" s="37" t="n"/>
+      <c r="K25" s="36" t="n"/>
+      <c r="L25" s="37" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="38" t="inlineStr">
@@ -2808,6 +2868,11 @@
       <c r="I28" s="43" t="n"/>
       <c r="J28" s="16" t="n"/>
       <c r="K28" s="15" t="n"/>
+      <c r="L28" s="59" t="inlineStr">
+        <is>
+          <t>V06</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="44" t="inlineStr">
@@ -2864,7 +2929,8 @@
       <c r="H30" s="36" t="n"/>
       <c r="I30" s="36" t="n"/>
       <c r="J30" s="36" t="n"/>
-      <c r="K30" s="37" t="n"/>
+      <c r="K30" s="36" t="n"/>
+      <c r="L30" s="37" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="38" t="inlineStr">
@@ -2949,6 +3015,11 @@
       <c r="I32" s="50" t="n"/>
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="22" t="n"/>
+      <c r="L32" s="61" t="inlineStr">
+        <is>
+          <t>V03, V04</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="38" t="inlineStr">
@@ -2991,6 +3062,11 @@
       <c r="I33" s="43" t="n"/>
       <c r="J33" s="16" t="n"/>
       <c r="K33" s="15" t="n"/>
+      <c r="L33" s="59" t="inlineStr">
+        <is>
+          <t>V11</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="44" t="inlineStr">
@@ -3075,6 +3151,11 @@
       <c r="I35" s="43" t="n"/>
       <c r="J35" s="16" t="n"/>
       <c r="K35" s="15" t="n"/>
+      <c r="L35" s="62" t="inlineStr">
+        <is>
+          <t>V09, V10</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="44" t="inlineStr">
@@ -3199,6 +3280,11 @@
       <c r="I38" s="50" t="n"/>
       <c r="J38" s="23" t="n"/>
       <c r="K38" s="22" t="n"/>
+      <c r="L38" s="61" t="inlineStr">
+        <is>
+          <t>V13, V14</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="38" t="inlineStr">
@@ -3295,7 +3381,8 @@
       <c r="H41" s="36" t="n"/>
       <c r="I41" s="36" t="n"/>
       <c r="J41" s="36" t="n"/>
-      <c r="K41" s="37" t="n"/>
+      <c r="K41" s="36" t="n"/>
+      <c r="L41" s="37" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="38" t="inlineStr">
@@ -3338,6 +3425,11 @@
       <c r="I42" s="43" t="n"/>
       <c r="J42" s="16" t="n"/>
       <c r="K42" s="15" t="n"/>
+      <c r="L42" s="59" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="44" t="inlineStr">
@@ -3380,6 +3472,11 @@
       <c r="I43" s="50" t="n"/>
       <c r="J43" s="23" t="n"/>
       <c r="K43" s="22" t="n"/>
+      <c r="L43" s="60" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
@@ -3422,6 +3519,11 @@
       <c r="I44" s="43" t="n"/>
       <c r="J44" s="16" t="n"/>
       <c r="K44" s="15" t="n"/>
+      <c r="L44" s="59" t="inlineStr">
+        <is>
+          <t>V03</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="44" t="inlineStr">
@@ -3464,6 +3566,11 @@
       <c r="I45" s="50" t="n"/>
       <c r="J45" s="23" t="n"/>
       <c r="K45" s="22" t="n"/>
+      <c r="L45" s="60" t="inlineStr">
+        <is>
+          <t>V04</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="38" t="inlineStr">
@@ -3506,6 +3613,11 @@
       <c r="I46" s="43" t="n"/>
       <c r="J46" s="16" t="n"/>
       <c r="K46" s="15" t="n"/>
+      <c r="L46" s="59" t="inlineStr">
+        <is>
+          <t>V05</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="44" t="inlineStr">
@@ -3548,6 +3660,11 @@
       <c r="I47" s="50" t="n"/>
       <c r="J47" s="23" t="n"/>
       <c r="K47" s="22" t="n"/>
+      <c r="L47" s="60" t="inlineStr">
+        <is>
+          <t>V06</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="38" t="inlineStr">
@@ -3590,6 +3707,11 @@
       <c r="I48" s="43" t="n"/>
       <c r="J48" s="16" t="n"/>
       <c r="K48" s="15" t="n"/>
+      <c r="L48" s="59" t="inlineStr">
+        <is>
+          <t>V09</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="44" t="inlineStr">
@@ -3632,6 +3754,11 @@
       <c r="I49" s="50" t="n"/>
       <c r="J49" s="23" t="n"/>
       <c r="K49" s="22" t="n"/>
+      <c r="L49" s="60" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="38" t="inlineStr">
@@ -3674,6 +3801,11 @@
       <c r="I50" s="43" t="n"/>
       <c r="J50" s="16" t="n"/>
       <c r="K50" s="15" t="n"/>
+      <c r="L50" s="59" t="inlineStr">
+        <is>
+          <t>V11</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="44" t="inlineStr">
@@ -3716,6 +3848,11 @@
       <c r="I51" s="50" t="n"/>
       <c r="J51" s="23" t="n"/>
       <c r="K51" s="22" t="n"/>
+      <c r="L51" s="60" t="inlineStr">
+        <is>
+          <t>V12</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="38" t="inlineStr">
@@ -3758,6 +3895,11 @@
       <c r="I52" s="43" t="n"/>
       <c r="J52" s="16" t="n"/>
       <c r="K52" s="15" t="n"/>
+      <c r="L52" s="59" t="inlineStr">
+        <is>
+          <t>V13</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="44" t="inlineStr">
@@ -3800,6 +3942,11 @@
       <c r="I53" s="50" t="n"/>
       <c r="J53" s="23" t="n"/>
       <c r="K53" s="22" t="n"/>
+      <c r="L53" s="60" t="inlineStr">
+        <is>
+          <t>V14</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="38" t="inlineStr">
@@ -3856,7 +4003,8 @@
       <c r="H55" s="36" t="n"/>
       <c r="I55" s="36" t="n"/>
       <c r="J55" s="36" t="n"/>
-      <c r="K55" s="37" t="n"/>
+      <c r="K55" s="36" t="n"/>
+      <c r="L55" s="37" t="n"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="38" t="inlineStr">
@@ -3979,6 +4127,11 @@
       <c r="I58" s="43" t="n"/>
       <c r="J58" s="16" t="n"/>
       <c r="K58" s="15" t="n"/>
+      <c r="L58" s="59" t="inlineStr">
+        <is>
+          <t>V17</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="44" t="inlineStr">
@@ -4021,6 +4174,11 @@
       <c r="I59" s="50" t="n"/>
       <c r="J59" s="23" t="n"/>
       <c r="K59" s="22" t="n"/>
+      <c r="L59" s="60" t="inlineStr">
+        <is>
+          <t>V17</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="38" t="inlineStr">
@@ -4063,6 +4221,11 @@
       <c r="I60" s="43" t="n"/>
       <c r="J60" s="16" t="n"/>
       <c r="K60" s="15" t="n"/>
+      <c r="L60" s="59" t="inlineStr">
+        <is>
+          <t>V17</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="35" t="inlineStr">
@@ -4079,7 +4242,8 @@
       <c r="H61" s="36" t="n"/>
       <c r="I61" s="36" t="n"/>
       <c r="J61" s="36" t="n"/>
-      <c r="K61" s="37" t="n"/>
+      <c r="K61" s="36" t="n"/>
+      <c r="L61" s="37" t="n"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="38" t="inlineStr">
@@ -4162,6 +4326,11 @@
       <c r="I63" s="50" t="n"/>
       <c r="J63" s="23" t="n"/>
       <c r="K63" s="22" t="n"/>
+      <c r="L63" s="60" t="inlineStr">
+        <is>
+          <t>V07</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="38" t="inlineStr">
@@ -4246,6 +4415,11 @@
       <c r="I65" s="50" t="n"/>
       <c r="J65" s="23" t="n"/>
       <c r="K65" s="22" t="n"/>
+      <c r="L65" s="61" t="inlineStr">
+        <is>
+          <t>V08, V09, V10, V11</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="38" t="inlineStr">
@@ -4330,6 +4504,11 @@
       <c r="I67" s="50" t="n"/>
       <c r="J67" s="23" t="n"/>
       <c r="K67" s="22" t="n"/>
+      <c r="L67" s="61" t="inlineStr">
+        <is>
+          <t>V07, V08, V15</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="38" t="inlineStr">
@@ -4374,6 +4553,11 @@
       <c r="I68" s="43" t="n"/>
       <c r="J68" s="16" t="n"/>
       <c r="K68" s="15" t="n"/>
+      <c r="L68" s="62" t="inlineStr">
+        <is>
+          <t>V07, V08, V09</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="44" t="inlineStr">
@@ -4416,6 +4600,11 @@
       <c r="I69" s="50" t="n"/>
       <c r="J69" s="23" t="n"/>
       <c r="K69" s="22" t="n"/>
+      <c r="L69" s="60" t="inlineStr">
+        <is>
+          <t>V15</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="38" t="inlineStr">
@@ -4500,6 +4689,11 @@
       <c r="I71" s="50" t="n"/>
       <c r="J71" s="23" t="n"/>
       <c r="K71" s="22" t="n"/>
+      <c r="L71" s="61" t="inlineStr">
+        <is>
+          <t>V07, V08, V14</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="38" t="inlineStr">
@@ -4542,6 +4736,11 @@
       <c r="I72" s="43" t="n"/>
       <c r="J72" s="16" t="n"/>
       <c r="K72" s="15" t="n"/>
+      <c r="L72" s="59" t="inlineStr">
+        <is>
+          <t>V16</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="44" t="inlineStr">
@@ -4586,6 +4785,11 @@
       <c r="I73" s="50" t="n"/>
       <c r="J73" s="23" t="n"/>
       <c r="K73" s="22" t="n"/>
+      <c r="L73" s="61" t="inlineStr">
+        <is>
+          <t>V07, V08</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="38" t="inlineStr">
@@ -4628,6 +4832,11 @@
       <c r="I74" s="43" t="n"/>
       <c r="J74" s="16" t="n"/>
       <c r="K74" s="15" t="n"/>
+      <c r="L74" s="59" t="inlineStr">
+        <is>
+          <t>V08</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="35" t="inlineStr">
@@ -4644,7 +4853,8 @@
       <c r="H75" s="36" t="n"/>
       <c r="I75" s="36" t="n"/>
       <c r="J75" s="36" t="n"/>
-      <c r="K75" s="37" t="n"/>
+      <c r="K75" s="36" t="n"/>
+      <c r="L75" s="37" t="n"/>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="38" t="inlineStr">
@@ -4689,6 +4899,11 @@
       <c r="I76" s="43" t="n"/>
       <c r="J76" s="16" t="n"/>
       <c r="K76" s="15" t="n"/>
+      <c r="L76" s="62" t="inlineStr">
+        <is>
+          <t>V07, V08, V15, V16, V17</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="44" t="inlineStr">
@@ -4773,6 +4988,11 @@
       <c r="I78" s="43" t="n"/>
       <c r="J78" s="16" t="n"/>
       <c r="K78" s="15" t="n"/>
+      <c r="L78" s="62" t="inlineStr">
+        <is>
+          <t>V07, V08, V15, V16, V17</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="44" t="inlineStr">
@@ -4857,6 +5077,11 @@
       <c r="I80" s="43" t="n"/>
       <c r="J80" s="16" t="n"/>
       <c r="K80" s="15" t="n"/>
+      <c r="L80" s="62" t="inlineStr">
+        <is>
+          <t>V07, V08, V15, V16, V17</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="44" t="inlineStr">
@@ -4953,7 +5178,8 @@
       <c r="H83" s="36" t="n"/>
       <c r="I83" s="36" t="n"/>
       <c r="J83" s="36" t="n"/>
-      <c r="K83" s="37" t="n"/>
+      <c r="K83" s="36" t="n"/>
+      <c r="L83" s="37" t="n"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="38" t="inlineStr">
@@ -13300,20 +13526,20 @@
       <c r="K600" s="53" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K600"/>
+  <autoFilter ref="A4:L600"/>
   <mergeCells count="12">
-    <mergeCell ref="A61:K61"/>
-    <mergeCell ref="A83:K83"/>
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="A55:K55"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A75:K75"/>
-    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A75:L75"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A55:L55"/>
+    <mergeCell ref="A83:L83"/>
+    <mergeCell ref="A30:L30"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A61:L61"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H600">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -13337,6 +13563,33 @@
       <formula1>"G0,G1,G2,G3,G4,G5,G6,G7,G8,G9"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId25"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>